<commit_message>
Removes outdated course docs and updates club constitution
Deletes legacy cryptography and identity management materials to streamline course content.

Updates MCCSVA constitution for clarity on officer eligibility, advisor responsibilities, and club policy alignment; revises language to reflect MCC-specific requirements.

Refreshes officer interest and club status spreadsheets to support current organization needs.
</commit_message>
<xml_diff>
--- a/McLennan-Community-College/_MCCSVA/Officer Interest Sheet.xlsx
+++ b/McLennan-Community-College/_MCCSVA/Officer Interest Sheet.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/d62837459e03f1f2/Documents/Github-Repo-for-Schools/McLennan-Community-College/_MCCSVA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10" documentId="11_6F4D07011E43C98649FB880530DD7AD9575B09A8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{936AE5B6-F6FF-4A11-B193-497051898351}"/>
+  <xr:revisionPtr revIDLastSave="16" documentId="11_6F4D07011E43C98649FB880530DD7AD9575B09A8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{101D57EC-78BD-4345-87B3-DCD01F6EA923}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -84,7 +84,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -207,11 +207,26 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
@@ -219,15 +234,18 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -465,24 +483,24 @@
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="B1" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="C1" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="D1" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="E1" s="6" t="s">
+      <c r="E1" s="8" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A2" s="7"/>
-      <c r="B2" s="8"/>
-      <c r="C2" s="8"/>
-      <c r="D2" s="8"/>
+      <c r="A2" s="5"/>
+      <c r="B2" s="7"/>
+      <c r="C2" s="7"/>
+      <c r="D2" s="7"/>
       <c r="E2" s="9"/>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
@@ -801,46 +819,46 @@
       <c r="E47" s="1"/>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A48" s="2"/>
-      <c r="B48" s="2"/>
-      <c r="C48" s="2"/>
-      <c r="D48" s="2"/>
-      <c r="E48" s="2"/>
+      <c r="A48" s="10"/>
+      <c r="B48" s="10"/>
+      <c r="C48" s="10"/>
+      <c r="D48" s="10"/>
+      <c r="E48" s="10"/>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A49" s="1"/>
-      <c r="B49" s="1"/>
-      <c r="C49" s="1"/>
-      <c r="D49" s="1"/>
-      <c r="E49" s="1"/>
+      <c r="A49" s="11"/>
+      <c r="B49" s="11"/>
+      <c r="C49" s="11"/>
+      <c r="D49" s="11"/>
+      <c r="E49" s="11"/>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A50" s="2"/>
-      <c r="B50" s="2"/>
-      <c r="C50" s="2"/>
-      <c r="D50" s="2"/>
-      <c r="E50" s="2"/>
+      <c r="A50" s="12"/>
+      <c r="B50" s="12"/>
+      <c r="C50" s="12"/>
+      <c r="D50" s="12"/>
+      <c r="E50" s="12"/>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A51" s="1"/>
-      <c r="B51" s="1"/>
-      <c r="C51" s="1"/>
-      <c r="D51" s="1"/>
-      <c r="E51" s="1"/>
+      <c r="A51" s="11"/>
+      <c r="B51" s="11"/>
+      <c r="C51" s="11"/>
+      <c r="D51" s="11"/>
+      <c r="E51" s="11"/>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A52" s="2"/>
-      <c r="B52" s="2"/>
-      <c r="C52" s="2"/>
-      <c r="D52" s="2"/>
-      <c r="E52" s="2"/>
+      <c r="A52" s="12"/>
+      <c r="B52" s="12"/>
+      <c r="C52" s="12"/>
+      <c r="D52" s="12"/>
+      <c r="E52" s="12"/>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A53" s="1"/>
-      <c r="B53" s="1"/>
-      <c r="C53" s="1"/>
-      <c r="D53" s="1"/>
-      <c r="E53" s="1"/>
+      <c r="A53" s="3"/>
+      <c r="B53" s="3"/>
+      <c r="C53" s="3"/>
+      <c r="D53" s="3"/>
+      <c r="E53" s="3"/>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A54" s="2"/>
@@ -893,17 +911,121 @@
     </row>
   </sheetData>
   <mergeCells count="150">
-    <mergeCell ref="B31:B32"/>
-    <mergeCell ref="B33:B34"/>
-    <mergeCell ref="B35:B36"/>
-    <mergeCell ref="B37:B38"/>
-    <mergeCell ref="B39:B40"/>
-    <mergeCell ref="B41:B42"/>
-    <mergeCell ref="B21:B22"/>
-    <mergeCell ref="B23:B24"/>
-    <mergeCell ref="B25:B26"/>
-    <mergeCell ref="B27:B28"/>
-    <mergeCell ref="B29:B30"/>
+    <mergeCell ref="C43:C44"/>
+    <mergeCell ref="D55:D56"/>
+    <mergeCell ref="D57:D58"/>
+    <mergeCell ref="D59:D60"/>
+    <mergeCell ref="E55:E56"/>
+    <mergeCell ref="E57:E58"/>
+    <mergeCell ref="E59:E60"/>
+    <mergeCell ref="E39:E40"/>
+    <mergeCell ref="E41:E42"/>
+    <mergeCell ref="D45:D46"/>
+    <mergeCell ref="D47:D48"/>
+    <mergeCell ref="D49:D50"/>
+    <mergeCell ref="D51:D52"/>
+    <mergeCell ref="D53:D54"/>
+    <mergeCell ref="D43:D44"/>
+    <mergeCell ref="D39:D40"/>
+    <mergeCell ref="D41:D42"/>
+    <mergeCell ref="E45:E46"/>
+    <mergeCell ref="E47:E48"/>
+    <mergeCell ref="E49:E50"/>
+    <mergeCell ref="E51:E52"/>
+    <mergeCell ref="E53:E54"/>
+    <mergeCell ref="E43:E44"/>
+    <mergeCell ref="C55:C56"/>
+    <mergeCell ref="D31:D32"/>
+    <mergeCell ref="D33:D34"/>
+    <mergeCell ref="E31:E32"/>
+    <mergeCell ref="E33:E34"/>
+    <mergeCell ref="C35:C36"/>
+    <mergeCell ref="C37:C38"/>
+    <mergeCell ref="D35:D36"/>
+    <mergeCell ref="D37:D38"/>
+    <mergeCell ref="E35:E36"/>
+    <mergeCell ref="E37:E38"/>
+    <mergeCell ref="C57:C58"/>
+    <mergeCell ref="B49:B50"/>
+    <mergeCell ref="B51:B52"/>
+    <mergeCell ref="B53:B54"/>
+    <mergeCell ref="B55:B56"/>
+    <mergeCell ref="B57:B58"/>
+    <mergeCell ref="B59:B60"/>
+    <mergeCell ref="C53:C54"/>
+    <mergeCell ref="C59:C60"/>
+    <mergeCell ref="C49:C50"/>
+    <mergeCell ref="C51:C52"/>
+    <mergeCell ref="A53:A54"/>
+    <mergeCell ref="A55:A56"/>
+    <mergeCell ref="A57:A58"/>
+    <mergeCell ref="A59:A60"/>
+    <mergeCell ref="A31:A32"/>
+    <mergeCell ref="A33:A34"/>
+    <mergeCell ref="A35:A36"/>
+    <mergeCell ref="A37:A38"/>
+    <mergeCell ref="A39:A40"/>
+    <mergeCell ref="A41:A42"/>
+    <mergeCell ref="A43:A44"/>
+    <mergeCell ref="A21:A22"/>
+    <mergeCell ref="A23:A24"/>
+    <mergeCell ref="A25:A26"/>
+    <mergeCell ref="A27:A28"/>
+    <mergeCell ref="A29:A30"/>
+    <mergeCell ref="A45:A46"/>
+    <mergeCell ref="A47:A48"/>
+    <mergeCell ref="A49:A50"/>
+    <mergeCell ref="A51:A52"/>
+    <mergeCell ref="E21:E22"/>
+    <mergeCell ref="E23:E24"/>
+    <mergeCell ref="E25:E26"/>
+    <mergeCell ref="E27:E28"/>
+    <mergeCell ref="E29:E30"/>
+    <mergeCell ref="E3:E4"/>
+    <mergeCell ref="E5:E6"/>
+    <mergeCell ref="E7:E8"/>
+    <mergeCell ref="E9:E10"/>
+    <mergeCell ref="E11:E12"/>
+    <mergeCell ref="E13:E14"/>
+    <mergeCell ref="E15:E16"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="B1:B2"/>
+    <mergeCell ref="C1:C2"/>
+    <mergeCell ref="D1:D2"/>
+    <mergeCell ref="E1:E2"/>
+    <mergeCell ref="B3:B4"/>
+    <mergeCell ref="B5:B6"/>
+    <mergeCell ref="E17:E18"/>
+    <mergeCell ref="E19:E20"/>
+    <mergeCell ref="A3:A4"/>
+    <mergeCell ref="A5:A6"/>
+    <mergeCell ref="A7:A8"/>
+    <mergeCell ref="A9:A10"/>
+    <mergeCell ref="A11:A12"/>
+    <mergeCell ref="A13:A14"/>
+    <mergeCell ref="A15:A16"/>
+    <mergeCell ref="A17:A18"/>
+    <mergeCell ref="A19:A20"/>
+    <mergeCell ref="B7:B8"/>
+    <mergeCell ref="B9:B10"/>
+    <mergeCell ref="B11:B12"/>
+    <mergeCell ref="B13:B14"/>
+    <mergeCell ref="B15:B16"/>
+    <mergeCell ref="B17:B18"/>
+    <mergeCell ref="D17:D18"/>
+    <mergeCell ref="D19:D20"/>
+    <mergeCell ref="D21:D22"/>
+    <mergeCell ref="D23:D24"/>
+    <mergeCell ref="D25:D26"/>
+    <mergeCell ref="D27:D28"/>
+    <mergeCell ref="D29:D30"/>
+    <mergeCell ref="D3:D4"/>
+    <mergeCell ref="D5:D6"/>
+    <mergeCell ref="D7:D8"/>
+    <mergeCell ref="D9:D10"/>
+    <mergeCell ref="D11:D12"/>
+    <mergeCell ref="D13:D14"/>
+    <mergeCell ref="D15:D16"/>
     <mergeCell ref="B45:B46"/>
     <mergeCell ref="B47:B48"/>
     <mergeCell ref="B43:B44"/>
@@ -928,125 +1050,21 @@
     <mergeCell ref="C29:C30"/>
     <mergeCell ref="C45:C46"/>
     <mergeCell ref="C47:C48"/>
-    <mergeCell ref="D17:D18"/>
-    <mergeCell ref="D19:D20"/>
-    <mergeCell ref="D21:D22"/>
-    <mergeCell ref="D23:D24"/>
-    <mergeCell ref="D25:D26"/>
-    <mergeCell ref="D27:D28"/>
-    <mergeCell ref="D29:D30"/>
-    <mergeCell ref="D3:D4"/>
-    <mergeCell ref="D5:D6"/>
-    <mergeCell ref="D7:D8"/>
-    <mergeCell ref="D9:D10"/>
-    <mergeCell ref="D11:D12"/>
-    <mergeCell ref="D13:D14"/>
-    <mergeCell ref="D15:D16"/>
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="B1:B2"/>
-    <mergeCell ref="C1:C2"/>
-    <mergeCell ref="D1:D2"/>
-    <mergeCell ref="E1:E2"/>
-    <mergeCell ref="B3:B4"/>
-    <mergeCell ref="B5:B6"/>
-    <mergeCell ref="E17:E18"/>
-    <mergeCell ref="E19:E20"/>
-    <mergeCell ref="A3:A4"/>
-    <mergeCell ref="A5:A6"/>
-    <mergeCell ref="A7:A8"/>
-    <mergeCell ref="A9:A10"/>
-    <mergeCell ref="A11:A12"/>
-    <mergeCell ref="A13:A14"/>
-    <mergeCell ref="A15:A16"/>
-    <mergeCell ref="A17:A18"/>
-    <mergeCell ref="A19:A20"/>
-    <mergeCell ref="B7:B8"/>
-    <mergeCell ref="B9:B10"/>
-    <mergeCell ref="B11:B12"/>
-    <mergeCell ref="B13:B14"/>
-    <mergeCell ref="B15:B16"/>
-    <mergeCell ref="B17:B18"/>
-    <mergeCell ref="E21:E22"/>
-    <mergeCell ref="E23:E24"/>
-    <mergeCell ref="E25:E26"/>
-    <mergeCell ref="E27:E28"/>
-    <mergeCell ref="E29:E30"/>
-    <mergeCell ref="E3:E4"/>
-    <mergeCell ref="E5:E6"/>
-    <mergeCell ref="E7:E8"/>
-    <mergeCell ref="E9:E10"/>
-    <mergeCell ref="E11:E12"/>
-    <mergeCell ref="E13:E14"/>
-    <mergeCell ref="E15:E16"/>
-    <mergeCell ref="A21:A22"/>
-    <mergeCell ref="A23:A24"/>
-    <mergeCell ref="A25:A26"/>
-    <mergeCell ref="A27:A28"/>
-    <mergeCell ref="A29:A30"/>
-    <mergeCell ref="A45:A46"/>
-    <mergeCell ref="A47:A48"/>
-    <mergeCell ref="A49:A50"/>
-    <mergeCell ref="A51:A52"/>
-    <mergeCell ref="A53:A54"/>
-    <mergeCell ref="A55:A56"/>
-    <mergeCell ref="A57:A58"/>
-    <mergeCell ref="A59:A60"/>
-    <mergeCell ref="A31:A32"/>
-    <mergeCell ref="A33:A34"/>
-    <mergeCell ref="A35:A36"/>
-    <mergeCell ref="A37:A38"/>
-    <mergeCell ref="A39:A40"/>
-    <mergeCell ref="A41:A42"/>
-    <mergeCell ref="A43:A44"/>
-    <mergeCell ref="C57:C58"/>
-    <mergeCell ref="B49:B50"/>
-    <mergeCell ref="B51:B52"/>
-    <mergeCell ref="B53:B54"/>
-    <mergeCell ref="B55:B56"/>
-    <mergeCell ref="B57:B58"/>
-    <mergeCell ref="B59:B60"/>
-    <mergeCell ref="C53:C54"/>
-    <mergeCell ref="C59:C60"/>
-    <mergeCell ref="C49:C50"/>
-    <mergeCell ref="C51:C52"/>
-    <mergeCell ref="D31:D32"/>
-    <mergeCell ref="D33:D34"/>
-    <mergeCell ref="E31:E32"/>
-    <mergeCell ref="E33:E34"/>
-    <mergeCell ref="C35:C36"/>
-    <mergeCell ref="C37:C38"/>
-    <mergeCell ref="D35:D36"/>
-    <mergeCell ref="D37:D38"/>
-    <mergeCell ref="E35:E36"/>
-    <mergeCell ref="E37:E38"/>
-    <mergeCell ref="C43:C44"/>
-    <mergeCell ref="D55:D56"/>
-    <mergeCell ref="D57:D58"/>
-    <mergeCell ref="D59:D60"/>
-    <mergeCell ref="E55:E56"/>
-    <mergeCell ref="E57:E58"/>
-    <mergeCell ref="E59:E60"/>
-    <mergeCell ref="E39:E40"/>
-    <mergeCell ref="E41:E42"/>
-    <mergeCell ref="D45:D46"/>
-    <mergeCell ref="D47:D48"/>
-    <mergeCell ref="D49:D50"/>
-    <mergeCell ref="D51:D52"/>
-    <mergeCell ref="D53:D54"/>
-    <mergeCell ref="D43:D44"/>
-    <mergeCell ref="D39:D40"/>
-    <mergeCell ref="D41:D42"/>
-    <mergeCell ref="E45:E46"/>
-    <mergeCell ref="E47:E48"/>
-    <mergeCell ref="E49:E50"/>
-    <mergeCell ref="E51:E52"/>
-    <mergeCell ref="E53:E54"/>
-    <mergeCell ref="E43:E44"/>
-    <mergeCell ref="C55:C56"/>
+    <mergeCell ref="B31:B32"/>
+    <mergeCell ref="B33:B34"/>
+    <mergeCell ref="B35:B36"/>
+    <mergeCell ref="B37:B38"/>
+    <mergeCell ref="B39:B40"/>
+    <mergeCell ref="B41:B42"/>
+    <mergeCell ref="B21:B22"/>
+    <mergeCell ref="B23:B24"/>
+    <mergeCell ref="B25:B26"/>
+    <mergeCell ref="B27:B28"/>
+    <mergeCell ref="B29:B30"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup scale="65" fitToHeight="0" orientation="landscape" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
+  <pageSetup scale="63" fitToHeight="0" orientation="landscape" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
   <headerFooter>
     <oddHeader>&amp;L&amp;"-,Bold"&amp;12MCCSVA Officer Interest Sheet&amp;C&amp;12&amp;D</oddHeader>
     <oddFooter>&amp;L&amp;"-,Bold"&amp;14Eligibility Checklist:&amp;"-,Regular"&amp;10

</xml_diff>